<commit_message>
Chap 6, EX 21
</commit_message>
<xml_diff>
--- a/Chapter6_Study_Checkin_Record_English_One_Exercise_Per_Day.xlsx
+++ b/Chapter6_Study_Checkin_Record_English_One_Exercise_Per_Day.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="19935" windowHeight="7785" activeTab="3"/>
+    <workbookView windowWidth="19935" windowHeight="7785" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="Dashboard" sheetId="1" r:id="rId1"/>
@@ -894,13 +894,13 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="7">
+    <numFmt numFmtId="176" formatCode="yyyy\-mm\-dd"/>
     <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="176" formatCode="0.0%"/>
-    <numFmt numFmtId="177" formatCode="yyyy\-mm\-dd"/>
-    <numFmt numFmtId="178" formatCode="yyyy\-mm\-dd\ hh:mm"/>
+    <numFmt numFmtId="177" formatCode="yyyy\-mm\-dd\ hh:mm"/>
+    <numFmt numFmtId="178" formatCode="0.0%"/>
   </numFmts>
   <fonts count="30">
     <font>
@@ -950,6 +950,13 @@
     </font>
     <font>
       <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <color rgb="FF666666"/>
       <name val="Calibri"/>
       <charset val="134"/>
@@ -964,13 +971,6 @@
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="0"/>
-      <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
@@ -983,46 +983,8 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF0000FF"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="18"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="15"/>
+      <sz val="13"/>
       <color theme="3"/>
       <name val="Calibri"/>
       <charset val="134"/>
@@ -1037,14 +999,21 @@
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FF9C6500"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
-      <sz val="11"/>
+      <sz val="15"/>
       <color theme="3"/>
       <name val="Calibri"/>
       <charset val="134"/>
@@ -1067,7 +1036,54 @@
     <font>
       <b/>
       <sz val="11"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF0000FF"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <color rgb="FFFA7D00"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF7F7F7F"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF800080"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -1081,32 +1097,16 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <u/>
       <sz val="11"/>
-      <color rgb="FF800080"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
+      <color rgb="FF9C6500"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
-      <sz val="13"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
       <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -1176,7 +1176,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
+        <fgColor theme="8" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1188,121 +1194,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1320,7 +1212,133 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1338,25 +1356,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
+        <fgColor rgb="FFFFEB9C"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1407,20 +1407,24 @@
     <border>
       <left/>
       <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
-      <bottom style="double">
+      <top/>
+      <bottom style="medium">
         <color theme="4"/>
       </bottom>
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4"/>
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB2B2B2"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB2B2B2"/>
       </bottom>
       <diagonal/>
     </border>
@@ -1440,17 +1444,20 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color rgb="FFB2B2B2"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB2B2B2"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB2B2B2"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB2B2B2"/>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
       </bottom>
       <diagonal/>
     </border>
@@ -1472,169 +1479,162 @@
     <border>
       <left/>
       <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
       <bottom style="double">
-        <color rgb="FFFF8001"/>
+        <color theme="4"/>
       </bottom>
       <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="42" fontId="9" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="24" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="17" fillId="24" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="44" fontId="9" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="41" fontId="9" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="15" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="43" fontId="9" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="9" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="34" borderId="7" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="23" borderId="5" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="35" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="35" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="29" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="12" borderId="3" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="29" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="11" borderId="3" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="27" fillId="40" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="40" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -1643,7 +1643,7 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="49" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="177" fontId="4" fillId="3" borderId="1" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="176" fontId="4" fillId="3" borderId="1" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="1" fontId="5" fillId="4" borderId="1" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1658,10 +1658,10 @@
     <xf numFmtId="1" fontId="6" fillId="4" borderId="1" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="49" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="49" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="49" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="49" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="49" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1670,7 +1670,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="49" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="0" xfId="49" applyFont="1" applyFill="1"/>
     <xf numFmtId="49" fontId="5" fillId="4" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="49" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1678,58 +1678,58 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="49" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="49" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="49" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="49" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="49" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="49" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="177" fontId="5" fillId="4" borderId="1" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="176" fontId="5" fillId="4" borderId="1" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" xfId="49" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="1" xfId="49" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" xfId="49" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="6" borderId="1" xfId="49" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="49" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="178" fontId="0" fillId="3" borderId="1" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="177" fontId="7" fillId="3" borderId="1" xfId="49" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="178" fontId="0" fillId="6" borderId="1" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="177" fontId="7" fillId="6" borderId="1" xfId="49" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="1" fontId="6" fillId="6" borderId="1" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="49" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="49" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="177" fontId="6" fillId="4" borderId="1" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="176" fontId="6" fillId="4" borderId="1" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="49" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="49" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="49" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="1" xfId="49" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="49" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" xfId="49" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="49" applyFont="1" applyFill="1"/>
-    <xf numFmtId="177" fontId="4" fillId="3" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="176" fontId="4" fillId="3" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="8" borderId="0" xfId="49" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="49" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="49" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="9" borderId="0" xfId="49" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="9" borderId="0" xfId="49" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="6" fillId="4" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1738,22 +1738,22 @@
     <xf numFmtId="1" fontId="6" fillId="4" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="176" fontId="6" fillId="9" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="178" fontId="6" fillId="9" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="49" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="49" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="8" borderId="0" xfId="49" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="49" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="1" xfId="49" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="49" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="49" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="49" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="1" xfId="49" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2464,7 +2464,7 @@
       </c>
       <c r="D4" s="38">
         <f>COUNTIFS('Unit Plan'!R5:R48,"&gt;0",'Unit Plan'!S5:S48,"&lt;&gt;Yes")</f>
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="5" ht="24" customHeight="1" spans="1:4">
@@ -2489,7 +2489,7 @@
       </c>
       <c r="B6" s="38">
         <f>COUNTIF('Unit Plan'!Q5:Q48,"Completed")</f>
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="C6" s="36" t="s">
         <v>9</v>
@@ -2512,7 +2512,7 @@
       </c>
       <c r="D7" s="38">
         <f>IFERROR(AVERAGE('Unit Plan'!P5:P48),"")</f>
-        <v>300.000000003492</v>
+        <v>279.99999996624</v>
       </c>
     </row>
     <row r="8" ht="24" customHeight="1" spans="1:4">
@@ -2521,14 +2521,14 @@
       </c>
       <c r="B8" s="38">
         <f>COUNTIFS('Unit Plan'!C5:C48,"Exercise",'Unit Plan'!O5:O48,"&lt;&gt;")</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C8" s="36" t="s">
         <v>13</v>
       </c>
       <c r="D8" s="38">
         <f>COUNTIF('Daily Log'!A5:A64,"&lt;&gt;")</f>
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="9" ht="24" customHeight="1" spans="1:4">
@@ -2553,7 +2553,7 @@
       </c>
       <c r="B10" s="39">
         <f>IF(B5=0,"",B6/B5)</f>
-        <v>0.136363636363636</v>
+        <v>0.204545454545455</v>
       </c>
       <c r="C10" s="36" t="s">
         <v>17</v>
@@ -2636,7 +2636,7 @@
       </c>
       <c r="C17" s="43">
         <f>COUNTIFS('Unit Plan'!C5:C28,"Exercise",'Unit Plan'!Q5:Q28,"Completed")</f>
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D17" s="44" t="s">
         <v>28</v>
@@ -3187,7 +3187,7 @@
       </c>
       <c r="P9" s="8">
         <f t="shared" si="1"/>
-        <v>480.000000003492</v>
+        <v>479.999999951106</v>
       </c>
       <c r="Q9" s="30" t="s">
         <v>21</v>
@@ -3247,7 +3247,7 @@
       </c>
       <c r="P10" s="8">
         <f t="shared" si="1"/>
-        <v>120.000000003492</v>
+        <v>119.999999951106</v>
       </c>
       <c r="Q10" s="30" t="s">
         <v>21</v>
@@ -3306,7 +3306,7 @@
         <v/>
       </c>
       <c r="Q11" s="30" t="s">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="R11" s="28" t="str">
         <f t="shared" si="2"/>
@@ -3355,18 +3355,22 @@
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="N12" s="24"/>
-      <c r="O12" s="24"/>
-      <c r="P12" s="8" t="str">
+      <c r="N12" s="24">
+        <v>46121.5833333333</v>
+      </c>
+      <c r="O12" s="24">
+        <v>46121.75</v>
+      </c>
+      <c r="P12" s="8">
         <f t="shared" si="1"/>
-        <v/>
+        <v>239.999999996508</v>
       </c>
       <c r="Q12" s="30" t="s">
-        <v>30</v>
-      </c>
-      <c r="R12" s="28" t="str">
+        <v>21</v>
+      </c>
+      <c r="R12" s="28">
         <f t="shared" si="2"/>
-        <v/>
+        <v>46123</v>
       </c>
       <c r="S12" s="27" t="s">
         <v>82</v>
@@ -3418,7 +3422,7 @@
         <v/>
       </c>
       <c r="Q13" s="30" t="s">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="R13" s="28" t="str">
         <f t="shared" si="2"/>
@@ -5548,7 +5552,7 @@
         <v>91</v>
       </c>
       <c r="G6" s="11" t="s">
-        <v>82</v>
+        <v>244</v>
       </c>
     </row>
     <row r="7" ht="30" spans="1:7">
@@ -5571,7 +5575,7 @@
         <v>91</v>
       </c>
       <c r="G7" s="11" t="s">
-        <v>82</v>
+        <v>244</v>
       </c>
     </row>
     <row r="8" ht="30" spans="1:7">
@@ -6354,10 +6358,12 @@
       <c r="J7" s="6"/>
     </row>
     <row r="8" spans="1:10">
-      <c r="A8" s="4"/>
-      <c r="B8" s="5" t="str">
+      <c r="A8" s="4">
+        <v>46119</v>
+      </c>
+      <c r="B8" s="5">
         <f>IF(A8="","",A8-Protocol!$B$3+1)</f>
-        <v/>
+        <v>6</v>
       </c>
       <c r="C8" s="6"/>
       <c r="D8" s="7"/>
@@ -6372,10 +6378,12 @@
       <c r="J8" s="6"/>
     </row>
     <row r="9" spans="1:10">
-      <c r="A9" s="4"/>
-      <c r="B9" s="5" t="str">
+      <c r="A9" s="4">
+        <v>46120</v>
+      </c>
+      <c r="B9" s="5">
         <f>IF(A9="","",A9-Protocol!$B$3+1)</f>
-        <v/>
+        <v>7</v>
       </c>
       <c r="C9" s="6"/>
       <c r="D9" s="7"/>
@@ -6390,10 +6398,12 @@
       <c r="J9" s="6"/>
     </row>
     <row r="10" spans="1:10">
-      <c r="A10" s="4"/>
-      <c r="B10" s="5" t="str">
+      <c r="A10" s="4">
+        <v>46121</v>
+      </c>
+      <c r="B10" s="5">
         <f>IF(A10="","",A10-Protocol!$B$3+1)</f>
-        <v/>
+        <v>8</v>
       </c>
       <c r="C10" s="6"/>
       <c r="D10" s="7"/>

</xml_diff>

<commit_message>
Chap 6, summary 1
</commit_message>
<xml_diff>
--- a/Chapter6_Study_Checkin_Record_English_One_Exercise_Per_Day.xlsx
+++ b/Chapter6_Study_Checkin_Record_English_One_Exercise_Per_Day.xlsx
@@ -894,11 +894,11 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="7">
-    <numFmt numFmtId="176" formatCode="yyyy\-mm\-dd"/>
-    <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="176" formatCode="yyyy\-mm\-dd"/>
     <numFmt numFmtId="177" formatCode="yyyy\-mm\-dd\ hh:mm"/>
     <numFmt numFmtId="178" formatCode="0.0%"/>
   </numFmts>
@@ -969,15 +969,21 @@
     </font>
     <font>
       <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
       <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
+      <color rgb="FF006100"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -998,8 +1004,9 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
       <sz val="11"/>
-      <color theme="0"/>
+      <color rgb="FFFA7D00"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -1007,6 +1014,13 @@
     <font>
       <sz val="11"/>
       <color rgb="FF9C0006"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -1020,15 +1034,9 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
       <sz val="11"/>
-      <color rgb="FF3F3F76"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
+      <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -1059,7 +1067,14 @@
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FFFA7D00"/>
+      <color rgb="FF3F3F76"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C6500"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -1067,7 +1082,7 @@
     <font>
       <b/>
       <sz val="11"/>
-      <color rgb="FFFA7D00"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -1092,21 +1107,6 @@
       <b/>
       <sz val="11"/>
       <color rgb="FF3F3F3F"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C6500"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -1176,7 +1176,163 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor theme="8" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1188,79 +1344,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
+        <fgColor theme="9" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1273,90 +1357,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1390,41 +1390,11 @@
       <diagonal/>
     </border>
     <border>
-      <left style="double">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="double">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="double">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left/>
       <right/>
       <top/>
       <bottom style="medium">
         <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FFB2B2B2"/>
-      </left>
-      <right style="thin">
-        <color rgb="FFB2B2B2"/>
-      </right>
-      <top style="thin">
-        <color rgb="FFB2B2B2"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB2B2B2"/>
       </bottom>
       <diagonal/>
     </border>
@@ -1447,6 +1417,45 @@
       <left/>
       <right/>
       <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB2B2B2"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB2B2B2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
       <bottom style="medium">
         <color theme="4" tint="0.499984740745262"/>
       </bottom>
@@ -1455,9 +1464,11 @@
     <border>
       <left/>
       <right/>
-      <top/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
       <bottom style="double">
-        <color rgb="FFFF8001"/>
+        <color theme="4"/>
       </bottom>
       <diagonal/>
     </border>
@@ -1476,27 +1487,16 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
-      <bottom style="double">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="24" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="31" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1505,133 +1505,133 @@
     <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="16" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="25" borderId="6" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="23" borderId="5" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="28" fillId="17" borderId="10" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="15" fillId="17" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="29" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="35" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="12" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="35" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="12" borderId="3" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="40" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="40" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
@@ -2464,7 +2464,7 @@
       </c>
       <c r="D4" s="38">
         <f>COUNTIFS('Unit Plan'!R5:R48,"&gt;0",'Unit Plan'!S5:S48,"&lt;&gt;Yes")</f>
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
     <row r="5" ht="24" customHeight="1" spans="1:4">
@@ -2489,7 +2489,7 @@
       </c>
       <c r="B6" s="38">
         <f>COUNTIF('Unit Plan'!Q5:Q48,"Completed")</f>
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="C6" s="36" t="s">
         <v>9</v>
@@ -2512,7 +2512,7 @@
       </c>
       <c r="D7" s="38">
         <f>IFERROR(AVERAGE('Unit Plan'!P5:P48),"")</f>
-        <v>279.99999996624</v>
+        <v>743.999999990221</v>
       </c>
     </row>
     <row r="8" ht="24" customHeight="1" spans="1:4">
@@ -2521,7 +2521,7 @@
       </c>
       <c r="B8" s="38">
         <f>COUNTIFS('Unit Plan'!C5:C48,"Exercise",'Unit Plan'!O5:O48,"&lt;&gt;")</f>
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C8" s="36" t="s">
         <v>13</v>
@@ -2553,7 +2553,7 @@
       </c>
       <c r="B10" s="39">
         <f>IF(B5=0,"",B6/B5)</f>
-        <v>0.204545454545455</v>
+        <v>0.25</v>
       </c>
       <c r="C10" s="36" t="s">
         <v>17</v>
@@ -2636,7 +2636,7 @@
       </c>
       <c r="C17" s="43">
         <f>COUNTIFS('Unit Plan'!C5:C28,"Exercise",'Unit Plan'!Q5:Q28,"Completed")</f>
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D17" s="44" t="s">
         <v>28</v>
@@ -3363,7 +3363,7 @@
       </c>
       <c r="P12" s="8">
         <f t="shared" si="1"/>
-        <v>239.999999996508</v>
+        <v>240.000000048894</v>
       </c>
       <c r="Q12" s="30" t="s">
         <v>21</v>
@@ -3471,18 +3471,22 @@
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="N14" s="24"/>
-      <c r="O14" s="24"/>
-      <c r="P14" s="8" t="str">
+      <c r="N14" s="24">
+        <v>46123</v>
+      </c>
+      <c r="O14" s="24">
+        <v>46123</v>
+      </c>
+      <c r="P14" s="8">
         <f t="shared" si="1"/>
-        <v/>
+        <v>0</v>
       </c>
       <c r="Q14" s="30" t="s">
-        <v>30</v>
-      </c>
-      <c r="R14" s="28" t="str">
+        <v>21</v>
+      </c>
+      <c r="R14" s="28">
         <f t="shared" si="2"/>
-        <v/>
+        <v>46125</v>
       </c>
       <c r="S14" s="27" t="s">
         <v>82</v>
@@ -3527,18 +3531,22 @@
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="N15" s="24"/>
-      <c r="O15" s="24"/>
-      <c r="P15" s="8" t="str">
+      <c r="N15" s="24">
+        <v>46124</v>
+      </c>
+      <c r="O15" s="24">
+        <v>46126</v>
+      </c>
+      <c r="P15" s="8">
         <f t="shared" si="1"/>
-        <v/>
+        <v>2880</v>
       </c>
       <c r="Q15" s="30" t="s">
-        <v>30</v>
-      </c>
-      <c r="R15" s="28" t="str">
+        <v>21</v>
+      </c>
+      <c r="R15" s="28">
         <f t="shared" si="2"/>
-        <v/>
+        <v>46128</v>
       </c>
       <c r="S15" s="27" t="s">
         <v>82</v>

</xml_diff>

<commit_message>
Chap 6, EX 6
</commit_message>
<xml_diff>
--- a/Chapter6_Study_Checkin_Record_English_One_Exercise_Per_Day.xlsx
+++ b/Chapter6_Study_Checkin_Record_English_One_Exercise_Per_Day.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/737d3273260deef1/learning_notes/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="16" documentId="11_01F34EFC9B3AEB9EA895230763713F60C8048F18" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{44A05CAB-D096-4462-BEED-451A2F25D36A}"/>
+  <xr:revisionPtr revIDLastSave="22" documentId="11_01F34EFC9B3AEB9EA895230763713F60C8048F18" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5FA26B89-5CB0-4524-B8A7-5EE9E51D729E}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1924,7 +1924,7 @@
       </c>
       <c r="D4" s="34">
         <f>COUNTIFS('Unit Plan'!R5:R48,"&gt;0",'Unit Plan'!S5:S48,"&lt;&gt;Yes")</f>
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.25">
@@ -1949,7 +1949,7 @@
       </c>
       <c r="B6" s="34">
         <f>COUNTIF('Unit Plan'!Q5:Q48,"Completed")</f>
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C6" s="32" t="s">
         <v>9</v>
@@ -1972,7 +1972,7 @@
       </c>
       <c r="D7" s="34">
         <f>IFERROR(AVERAGE('Unit Plan'!P5:P48),"")</f>
-        <v>531.42857142158653</v>
+        <v>573.33333332790062</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.25">
@@ -1981,7 +1981,7 @@
       </c>
       <c r="B8" s="34">
         <f>COUNTIFS('Unit Plan'!C5:C48,"Exercise",'Unit Plan'!O5:O48,"&lt;&gt;")</f>
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C8" s="32" t="s">
         <v>13</v>
@@ -2013,7 +2013,7 @@
       </c>
       <c r="B10" s="35">
         <f>IF(B5=0,"",B6/B5)</f>
-        <v>0.45454545454545453</v>
+        <v>0.47727272727272729</v>
       </c>
       <c r="C10" s="32" t="s">
         <v>17</v>
@@ -2099,7 +2099,7 @@
       </c>
       <c r="C17" s="38">
         <f>COUNTIFS('Unit Plan'!C5:C28,"Exercise",'Unit Plan'!Q5:Q28,"Completed")</f>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D17" s="39" t="s">
         <v>28</v>
@@ -3671,18 +3671,22 @@
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="N25" s="22"/>
-      <c r="O25" s="22"/>
-      <c r="P25" s="6" t="str">
+      <c r="N25" s="22">
+        <v>46145</v>
+      </c>
+      <c r="O25" s="22">
+        <v>46145</v>
+      </c>
+      <c r="P25" s="6">
         <f t="shared" si="1"/>
-        <v/>
+        <v>0</v>
       </c>
       <c r="Q25" s="28" t="s">
-        <v>30</v>
-      </c>
-      <c r="R25" s="26" t="str">
+        <v>21</v>
+      </c>
+      <c r="R25" s="26">
         <f t="shared" si="2"/>
-        <v/>
+        <v>46147</v>
       </c>
       <c r="S25" s="25" t="s">
         <v>82</v>
@@ -3727,18 +3731,22 @@
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="N26" s="22"/>
-      <c r="O26" s="22"/>
-      <c r="P26" s="6" t="str">
+      <c r="N26" s="22">
+        <v>46147</v>
+      </c>
+      <c r="O26" s="22">
+        <v>46148</v>
+      </c>
+      <c r="P26" s="6">
         <f t="shared" si="1"/>
-        <v/>
+        <v>1440</v>
       </c>
       <c r="Q26" s="28" t="s">
         <v>30</v>
       </c>
-      <c r="R26" s="26" t="str">
+      <c r="R26" s="26">
         <f t="shared" si="2"/>
-        <v/>
+        <v>46150</v>
       </c>
       <c r="S26" s="25" t="s">
         <v>82</v>

</xml_diff>

<commit_message>
Chap 6, Ex 3
</commit_message>
<xml_diff>
--- a/Chapter6_Study_Checkin_Record_English_One_Exercise_Per_Day.xlsx
+++ b/Chapter6_Study_Checkin_Record_English_One_Exercise_Per_Day.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/737d3273260deef1/learning_notes/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="22" documentId="11_01F34EFC9B3AEB9EA895230763713F60C8048F18" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5FA26B89-5CB0-4524-B8A7-5EE9E51D729E}"/>
+  <xr:revisionPtr revIDLastSave="3" documentId="11_1327E116937BED0EA895230763713F4036575F06" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{27086029-37F6-40A9-8D48-10F564391581}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -914,8 +914,8 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="3">
     <numFmt numFmtId="176" formatCode="yyyy\-mm\-dd"/>
-    <numFmt numFmtId="177" formatCode="yyyy\-mm\-dd\ hh:mm"/>
-    <numFmt numFmtId="178" formatCode="0.0%"/>
+    <numFmt numFmtId="179" formatCode="yyyy\-mm\-dd\ hh:mm"/>
+    <numFmt numFmtId="180" formatCode="0.0%"/>
   </numFmts>
   <fonts count="12" x14ac:knownFonts="1">
     <font>
@@ -1146,13 +1146,13 @@
     <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="177" fontId="7" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="7" fillId="6" borderId="1" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="179" fontId="7" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="1" fontId="6" fillId="6" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="7" fillId="6" borderId="1" xfId="1" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1181,7 +1181,7 @@
     <xf numFmtId="1" fontId="6" fillId="4" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="178" fontId="6" fillId="9" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="180" fontId="6" fillId="9" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1" applyAlignment="1">
@@ -1202,10 +1202,10 @@
     <xf numFmtId="0" fontId="3" fillId="8" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="0" xfId="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="1" xr:uid="{00000000-0005-0000-0000-000031000000}"/>
@@ -1623,10 +1623,6 @@
 </xdr:wsDr>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="UnitPlanTable" displayName="UnitPlanTable" ref="A4:V48">
   <autoFilter ref="A4:V48" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
@@ -1924,7 +1920,7 @@
       </c>
       <c r="D4" s="34">
         <f>COUNTIFS('Unit Plan'!R5:R48,"&gt;0",'Unit Plan'!S5:S48,"&lt;&gt;Yes")</f>
-        <v>9</v>
+        <v>11</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.25">
@@ -1949,7 +1945,7 @@
       </c>
       <c r="B6" s="34">
         <f>COUNTIF('Unit Plan'!Q5:Q48,"Completed")</f>
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="C6" s="32" t="s">
         <v>9</v>
@@ -1972,7 +1968,7 @@
       </c>
       <c r="D7" s="34">
         <f>IFERROR(AVERAGE('Unit Plan'!P5:P48),"")</f>
-        <v>573.33333332790062</v>
+        <v>338.18181817737326</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.25">
@@ -1981,7 +1977,7 @@
       </c>
       <c r="B8" s="34">
         <f>COUNTIFS('Unit Plan'!C5:C48,"Exercise",'Unit Plan'!O5:O48,"&lt;&gt;")</f>
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="C8" s="32" t="s">
         <v>13</v>
@@ -2013,7 +2009,7 @@
       </c>
       <c r="B10" s="35">
         <f>IF(B5=0,"",B6/B5)</f>
-        <v>0.47727272727272729</v>
+        <v>0.54545454545454541</v>
       </c>
       <c r="C10" s="32" t="s">
         <v>17</v>
@@ -2099,7 +2095,7 @@
       </c>
       <c r="C17" s="38">
         <f>COUNTIFS('Unit Plan'!C5:C28,"Exercise",'Unit Plan'!Q5:Q28,"Completed")</f>
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="D17" s="39" t="s">
         <v>28</v>
@@ -2188,7 +2184,7 @@
       </c>
     </row>
     <row r="5" spans="1:11" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="45" t="s">
+      <c r="A5" s="44" t="s">
         <v>40</v>
       </c>
       <c r="B5" s="41"/>
@@ -2206,7 +2202,7 @@
       </c>
     </row>
     <row r="6" spans="1:11" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="44" t="s">
+      <c r="A6" s="45" t="s">
         <v>43</v>
       </c>
       <c r="B6" s="41"/>
@@ -2218,7 +2214,7 @@
       <c r="H6" s="41"/>
     </row>
     <row r="7" spans="1:11" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="44" t="s">
+      <c r="A7" s="45" t="s">
         <v>44</v>
       </c>
       <c r="B7" s="41"/>
@@ -2230,7 +2226,7 @@
       <c r="H7" s="41"/>
     </row>
     <row r="8" spans="1:11" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="44" t="s">
+      <c r="A8" s="45" t="s">
         <v>45</v>
       </c>
       <c r="B8" s="41"/>
@@ -2242,7 +2238,7 @@
       <c r="H8" s="41"/>
     </row>
     <row r="9" spans="1:11" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="44" t="s">
+      <c r="A9" s="45" t="s">
         <v>46</v>
       </c>
       <c r="B9" s="41"/>
@@ -2254,7 +2250,7 @@
       <c r="H9" s="41"/>
     </row>
     <row r="10" spans="1:11" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="44" t="s">
+      <c r="A10" s="45" t="s">
         <v>47</v>
       </c>
       <c r="B10" s="41"/>
@@ -2266,7 +2262,7 @@
       <c r="H10" s="41"/>
     </row>
     <row r="11" spans="1:11" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="44" t="s">
+      <c r="A11" s="45" t="s">
         <v>48</v>
       </c>
       <c r="B11" s="41"/>
@@ -2279,7 +2275,7 @@
     </row>
     <row r="12" spans="1:11" ht="21.95" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="13" spans="1:11" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="45" t="s">
+      <c r="A13" s="44" t="s">
         <v>49</v>
       </c>
       <c r="B13" s="41"/>
@@ -2291,7 +2287,7 @@
       <c r="H13" s="41"/>
     </row>
     <row r="14" spans="1:11" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="44" t="s">
+      <c r="A14" s="45" t="s">
         <v>50</v>
       </c>
       <c r="B14" s="41"/>
@@ -2303,7 +2299,7 @@
       <c r="H14" s="41"/>
     </row>
     <row r="15" spans="1:11" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="44" t="s">
+      <c r="A15" s="45" t="s">
         <v>51</v>
       </c>
       <c r="B15" s="41"/>
@@ -2315,7 +2311,7 @@
       <c r="H15" s="41"/>
     </row>
     <row r="16" spans="1:11" ht="21.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="44" t="s">
+      <c r="A16" s="45" t="s">
         <v>52</v>
       </c>
       <c r="B16" s="41"/>
@@ -2328,11 +2324,6 @@
     </row>
   </sheetData>
   <mergeCells count="12">
-    <mergeCell ref="A1:H1"/>
-    <mergeCell ref="A5:H5"/>
-    <mergeCell ref="A6:H6"/>
-    <mergeCell ref="A7:H7"/>
-    <mergeCell ref="A8:H8"/>
     <mergeCell ref="A15:H15"/>
     <mergeCell ref="A16:H16"/>
     <mergeCell ref="A9:H9"/>
@@ -2340,6 +2331,11 @@
     <mergeCell ref="A11:H11"/>
     <mergeCell ref="A13:H13"/>
     <mergeCell ref="A14:H14"/>
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A5:H5"/>
+    <mergeCell ref="A6:H6"/>
+    <mergeCell ref="A7:H7"/>
+    <mergeCell ref="A8:H8"/>
   </mergeCells>
   <phoneticPr fontId="11" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3161,7 +3157,7 @@
       </c>
       <c r="N16" s="22"/>
       <c r="O16" s="22"/>
-      <c r="P16" s="24" t="str">
+      <c r="P16" s="23" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
@@ -3735,18 +3731,18 @@
         <v>46147</v>
       </c>
       <c r="O26" s="22">
-        <v>46148</v>
+        <v>46147</v>
       </c>
       <c r="P26" s="6">
         <f t="shared" si="1"/>
-        <v>1440</v>
+        <v>0</v>
       </c>
       <c r="Q26" s="28" t="s">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="R26" s="26">
         <f t="shared" si="2"/>
-        <v>46150</v>
+        <v>46149</v>
       </c>
       <c r="S26" s="25" t="s">
         <v>82</v>
@@ -3791,18 +3787,22 @@
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="N27" s="22"/>
-      <c r="O27" s="22"/>
-      <c r="P27" s="6" t="str">
+      <c r="N27" s="22">
+        <v>46148</v>
+      </c>
+      <c r="O27" s="22">
+        <v>46148</v>
+      </c>
+      <c r="P27" s="6">
         <f t="shared" si="1"/>
-        <v/>
+        <v>0</v>
       </c>
       <c r="Q27" s="28" t="s">
-        <v>30</v>
-      </c>
-      <c r="R27" s="26" t="str">
+        <v>21</v>
+      </c>
+      <c r="R27" s="26">
         <f t="shared" si="2"/>
-        <v/>
+        <v>46150</v>
       </c>
       <c r="S27" s="25" t="s">
         <v>82</v>
@@ -3847,18 +3847,22 @@
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="N28" s="22"/>
-      <c r="O28" s="22"/>
-      <c r="P28" s="6" t="str">
+      <c r="N28" s="22">
+        <v>46149</v>
+      </c>
+      <c r="O28" s="22">
+        <v>46149</v>
+      </c>
+      <c r="P28" s="6">
         <f t="shared" si="1"/>
-        <v/>
+        <v>0</v>
       </c>
       <c r="Q28" s="28" t="s">
-        <v>30</v>
-      </c>
-      <c r="R28" s="26" t="str">
+        <v>21</v>
+      </c>
+      <c r="R28" s="26">
         <f t="shared" si="2"/>
-        <v/>
+        <v>46151</v>
       </c>
       <c r="S28" s="25" t="s">
         <v>82</v>
@@ -4967,9 +4971,9 @@
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="N48" s="23"/>
-      <c r="O48" s="23"/>
-      <c r="P48" s="24" t="str">
+      <c r="N48" s="24"/>
+      <c r="O48" s="24"/>
+      <c r="P48" s="23" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>

</xml_diff>

<commit_message>
Chap6, lots of Exs
</commit_message>
<xml_diff>
--- a/Chapter6_Study_Checkin_Record_English_One_Exercise_Per_Day.xlsx
+++ b/Chapter6_Study_Checkin_Record_English_One_Exercise_Per_Day.xlsx
@@ -894,15 +894,15 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="7">
+    <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="176" formatCode="yyyy\-mm\-dd\ hh:mm"/>
+    <numFmt numFmtId="177" formatCode="yyyy\-mm\-dd"/>
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="176" formatCode="0.0%"/>
-    <numFmt numFmtId="177" formatCode="yyyy\-mm\-dd"/>
-    <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="178" formatCode="yyyy\-mm\-dd\ hh:mm"/>
+    <numFmt numFmtId="178" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="30">
+  <fonts count="29">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -950,13 +950,6 @@
     </font>
     <font>
       <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
       <color rgb="FF666666"/>
       <name val="Calibri"/>
       <charset val="134"/>
@@ -968,24 +961,8 @@
       <charset val="134"/>
     </font>
     <font>
-      <b/>
-      <sz val="15"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <sz val="11"/>
-      <color rgb="FF3F3F76"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -999,78 +976,9 @@
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FF9C0006"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
       <color rgb="FFFA7D00"/>
       <name val="Calibri"/>
       <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF0000FF"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color rgb="FF800080"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="11"/>
-      <color rgb="FF7F7F7F"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -1090,10 +998,87 @@
     </font>
     <font>
       <b/>
+      <sz val="15"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="18"/>
       <color theme="3"/>
       <name val="Calibri"/>
       <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF0000FF"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF3F3F76"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF3F3F3F"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF7F7F7F"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF800080"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -1107,6 +1092,14 @@
       <b/>
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -1176,121 +1169,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1302,31 +1181,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.799981688894314"/>
+        <fgColor theme="6" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1344,7 +1199,127 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1357,6 +1332,24 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1393,6 +1386,15 @@
       <left/>
       <right/>
       <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
       <bottom style="medium">
         <color theme="4"/>
       </bottom>
@@ -1410,6 +1412,15 @@
       </top>
       <bottom style="thin">
         <color rgb="FFB2B2B2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
       </bottom>
       <diagonal/>
     </border>
@@ -1455,24 +1466,6 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="double">
-        <color rgb="FFFF8001"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left style="double">
         <color rgb="FF3F3F3F"/>
       </left>
@@ -1493,10 +1486,10 @@
     <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="11" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="26" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1505,136 +1498,136 @@
     <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="15" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="4" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="5" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="12" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="28" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="12" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="27" fillId="28" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="40" borderId="10" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="26" fillId="37" borderId="10" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="40" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="16" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -1658,10 +1651,10 @@
     <xf numFmtId="1" fontId="6" fillId="4" borderId="1" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="49" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="49" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="49" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="49" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="49" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1670,7 +1663,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="0" xfId="49" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="49" applyFont="1" applyFill="1"/>
     <xf numFmtId="49" fontId="5" fillId="4" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="49" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1678,10 +1671,10 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="49" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="49" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="49" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="49" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="49" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="49" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1690,46 +1683,46 @@
     <xf numFmtId="177" fontId="5" fillId="4" borderId="1" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="1" xfId="49" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" xfId="49" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="1" xfId="49" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" xfId="49" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="49" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="178" fontId="7" fillId="3" borderId="1" xfId="49" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="176" fontId="0" fillId="3" borderId="1" xfId="49" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="1" fontId="6" fillId="6" borderId="1" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="178" fontId="7" fillId="6" borderId="1" xfId="49" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="176" fontId="0" fillId="6" borderId="1" xfId="49" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="49" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="49" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="177" fontId="6" fillId="4" borderId="1" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="49" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="49" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="1" xfId="49" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="49" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" xfId="49" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="49" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="49" applyFont="1" applyFill="1"/>
     <xf numFmtId="177" fontId="4" fillId="3" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="8" borderId="0" xfId="49" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="49" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="49" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="9" borderId="0" xfId="49" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="0" xfId="49" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="6" fillId="4" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1738,22 +1731,22 @@
     <xf numFmtId="1" fontId="6" fillId="4" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="176" fontId="6" fillId="9" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="178" fontId="6" fillId="9" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="49" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="49" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="8" borderId="0" xfId="49" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="9" borderId="1" xfId="49" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="49" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="49" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="49" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="1" xfId="49" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="49" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2464,7 +2457,7 @@
       </c>
       <c r="D4" s="38">
         <f>COUNTIFS('Unit Plan'!R5:R48,"&gt;0",'Unit Plan'!S5:S48,"&lt;&gt;Yes")</f>
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="5" ht="24" customHeight="1" spans="1:4">
@@ -2489,7 +2482,7 @@
       </c>
       <c r="B6" s="38">
         <f>COUNTIF('Unit Plan'!Q5:Q48,"Completed")</f>
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C6" s="36" t="s">
         <v>9</v>
@@ -2512,7 +2505,7 @@
       </c>
       <c r="D7" s="38">
         <f>IFERROR(AVERAGE('Unit Plan'!P5:P48),"")</f>
-        <v>177.142857140529</v>
+        <v>169.090909088687</v>
       </c>
     </row>
     <row r="8" ht="24" customHeight="1" spans="1:4">
@@ -2521,7 +2514,7 @@
       </c>
       <c r="B8" s="38">
         <f>COUNTIFS('Unit Plan'!C5:C48,"Exercise",'Unit Plan'!O5:O48,"&lt;&gt;")</f>
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C8" s="36" t="s">
         <v>13</v>
@@ -2553,7 +2546,7 @@
       </c>
       <c r="B10" s="39">
         <f>IF(B5=0,"",B6/B5)</f>
-        <v>0.772727272727273</v>
+        <v>0.795454545454545</v>
       </c>
       <c r="C10" s="36" t="s">
         <v>17</v>
@@ -4943,18 +4936,22 @@
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="N39" s="24"/>
-      <c r="O39" s="24"/>
-      <c r="P39" s="8" t="str">
+      <c r="N39" s="24">
+        <v>46161</v>
+      </c>
+      <c r="O39" s="24">
+        <v>46161</v>
+      </c>
+      <c r="P39" s="8">
         <f t="shared" si="1"/>
-        <v/>
+        <v>0</v>
       </c>
       <c r="Q39" s="30" t="s">
-        <v>30</v>
-      </c>
-      <c r="R39" s="28" t="str">
+        <v>21</v>
+      </c>
+      <c r="R39" s="28">
         <f t="shared" si="2"/>
-        <v/>
+        <v>46163</v>
       </c>
       <c r="S39" s="27" t="s">
         <v>82</v>

</xml_diff>

<commit_message>
Chap 6, Ex 31
</commit_message>
<xml_diff>
--- a/Chapter6_Study_Checkin_Record_English_One_Exercise_Per_Day.xlsx
+++ b/Chapter6_Study_Checkin_Record_English_One_Exercise_Per_Day.xlsx
@@ -894,15 +894,15 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="7">
+    <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="176" formatCode="yyyy\-mm\-dd"/>
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="176" formatCode="yyyy\-mm\-dd\ hh:mm"/>
-    <numFmt numFmtId="177" formatCode="yyyy\-mm\-dd"/>
+    <numFmt numFmtId="177" formatCode="yyyy\-mm\-dd\ hh:mm"/>
     <numFmt numFmtId="178" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="30">
+  <fonts count="29">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -950,13 +950,6 @@
     </font>
     <font>
       <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
       <color rgb="FF666666"/>
       <name val="Calibri"/>
       <charset val="134"/>
@@ -968,39 +961,15 @@
       <charset val="134"/>
     </font>
     <font>
-      <b/>
       <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
+      <color theme="0"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FF9C0006"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -1015,7 +984,7 @@
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FF9C6500"/>
+      <color rgb="FF9C0006"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -1023,6 +992,14 @@
     <font>
       <sz val="11"/>
       <color rgb="FF006100"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -1053,21 +1030,52 @@
     </font>
     <font>
       <sz val="11"/>
+      <color rgb="FF9C6500"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <color rgb="FF3F3F76"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
       <sz val="11"/>
-      <color theme="0"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF3F3F3F"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
-      <color theme="1"/>
+      <color rgb="FFFA7D00"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -1089,24 +1097,9 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <b/>
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -1176,7 +1169,25 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1188,7 +1199,55 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFCC"/>
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1200,7 +1259,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
+        <fgColor theme="5"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1218,13 +1277,55 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor theme="7" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
+        <fgColor theme="8" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1242,121 +1343,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="4" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="FFA5A5A5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1390,41 +1383,11 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color rgb="FF7F7F7F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF7F7F7F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF7F7F7F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF7F7F7F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
       <left/>
       <right/>
       <top/>
       <bottom style="medium">
         <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
       </bottom>
       <diagonal/>
     </border>
@@ -1446,9 +1409,50 @@
     <border>
       <left/>
       <right/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
       <top/>
       <bottom style="medium">
         <color theme="4" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF7F7F7F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF7F7F7F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF7F7F7F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF7F7F7F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
       </bottom>
       <diagonal/>
     </border>
@@ -1476,27 +1480,16 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="4"/>
-      </top>
-      <bottom style="double">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="15" borderId="3" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="26" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1505,136 +1498,136 @@
     <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="12" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="4" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="12" borderId="6" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="29" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="29" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="27" fillId="40" borderId="10" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="10" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="10" borderId="3" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="13" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="32" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="28" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="40" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -1643,7 +1636,7 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="49" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="177" fontId="4" fillId="3" borderId="1" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="176" fontId="4" fillId="3" borderId="1" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="1" fontId="5" fillId="4" borderId="1" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1658,10 +1651,10 @@
     <xf numFmtId="1" fontId="6" fillId="4" borderId="1" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="49" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="49" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="49" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="49" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="49" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1670,7 +1663,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="0" xfId="49" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="49" applyFont="1" applyFill="1"/>
     <xf numFmtId="49" fontId="5" fillId="4" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="49" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1678,58 +1671,58 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="49" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="49" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="49" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="49" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="49" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="49" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="177" fontId="5" fillId="4" borderId="1" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="176" fontId="5" fillId="4" borderId="1" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="1" xfId="49" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" xfId="49" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="6" borderId="1" xfId="49" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" xfId="49" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="49" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="176" fontId="7" fillId="3" borderId="1" xfId="49" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="177" fontId="0" fillId="3" borderId="1" xfId="49" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="1" fontId="6" fillId="6" borderId="1" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="176" fontId="7" fillId="6" borderId="1" xfId="49" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="177" fontId="0" fillId="6" borderId="1" xfId="49" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="49" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="49" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="177" fontId="6" fillId="4" borderId="1" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="176" fontId="6" fillId="4" borderId="1" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="49" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="49" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="1" xfId="49" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="49" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" xfId="49" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="49" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="49" applyFont="1" applyFill="1"/>
-    <xf numFmtId="177" fontId="4" fillId="3" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="176" fontId="4" fillId="3" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="8" borderId="0" xfId="49" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="49" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="49" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="9" borderId="0" xfId="49" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="0" xfId="49" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="6" fillId="4" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1741,19 +1734,19 @@
     <xf numFmtId="178" fontId="6" fillId="9" borderId="0" xfId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="49" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="49" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="8" borderId="0" xfId="49" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="9" borderId="1" xfId="49" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="49" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="49" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="49" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="1" xfId="49" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="49" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2464,7 +2457,7 @@
       </c>
       <c r="D4" s="38">
         <f>COUNTIFS('Unit Plan'!R5:R48,"&gt;0",'Unit Plan'!S5:S48,"&lt;&gt;Yes")</f>
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="5" ht="24" customHeight="1" spans="1:4">
@@ -2489,7 +2482,7 @@
       </c>
       <c r="B6" s="38">
         <f>COUNTIF('Unit Plan'!Q5:Q48,"Completed")</f>
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C6" s="36" t="s">
         <v>9</v>
@@ -2512,7 +2505,7 @@
       </c>
       <c r="D7" s="38">
         <f>IFERROR(AVERAGE('Unit Plan'!P5:P48),"")</f>
-        <v>132.857142855397</v>
+        <v>177.931034481073</v>
       </c>
     </row>
     <row r="8" ht="24" customHeight="1" spans="1:4">
@@ -2521,7 +2514,7 @@
       </c>
       <c r="B8" s="38">
         <f>COUNTIFS('Unit Plan'!C5:C48,"Exercise",'Unit Plan'!O5:O48,"&lt;&gt;")</f>
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C8" s="36" t="s">
         <v>13</v>
@@ -2553,7 +2546,7 @@
       </c>
       <c r="B10" s="39">
         <f>IF(B5=0,"",B6/B5)</f>
-        <v>0.931818181818182</v>
+        <v>0.954545454545455</v>
       </c>
       <c r="C10" s="36" t="s">
         <v>17</v>
@@ -5363,18 +5356,22 @@
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="N46" s="24"/>
-      <c r="O46" s="24"/>
-      <c r="P46" s="8" t="str">
+      <c r="N46" s="24">
+        <v>46169</v>
+      </c>
+      <c r="O46" s="24">
+        <v>46170</v>
+      </c>
+      <c r="P46" s="8">
         <f t="shared" si="1"/>
-        <v/>
+        <v>1440</v>
       </c>
       <c r="Q46" s="30" t="s">
-        <v>30</v>
-      </c>
-      <c r="R46" s="28" t="str">
+        <v>21</v>
+      </c>
+      <c r="R46" s="28">
         <f t="shared" si="2"/>
-        <v/>
+        <v>46172</v>
       </c>
       <c r="S46" s="27" t="s">
         <v>82</v>
@@ -5521,11 +5518,11 @@
     <dataValidation type="list" allowBlank="1" sqref="Q5:Q48">
       <formula1>Protocol!$J$1:$J$5</formula1>
     </dataValidation>
+    <dataValidation type="list" allowBlank="1" sqref="T5:T48">
+      <formula1>Protocol!$K$1:$K$5</formula1>
+    </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="S5:S48">
       <formula1>"Yes,No"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="T5:T48">
-      <formula1>Protocol!$K$1:$K$5</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Chap 6, Ex 32, finished all exercises!
</commit_message>
<xml_diff>
--- a/Chapter6_Study_Checkin_Record_English_One_Exercise_Per_Day.xlsx
+++ b/Chapter6_Study_Checkin_Record_English_One_Exercise_Per_Day.xlsx
@@ -894,11 +894,11 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="7">
+    <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="42" formatCode="_ &quot;￥&quot;* #,##0_ ;_ &quot;￥&quot;* \-#,##0_ ;_ &quot;￥&quot;* &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="41" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
-    <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="176" formatCode="yyyy\-mm\-dd"/>
-    <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="177" formatCode="yyyy\-mm\-dd\ hh:mm"/>
     <numFmt numFmtId="178" formatCode="0.0%"/>
   </numFmts>
@@ -968,18 +968,18 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
+      <b/>
+      <sz val="13"/>
+      <color theme="3"/>
       <name val="Calibri"/>
-      <charset val="0"/>
+      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="15"/>
-      <color theme="3"/>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
       <name val="Calibri"/>
-      <charset val="134"/>
+      <charset val="0"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -990,8 +990,9 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
       <sz val="11"/>
-      <color rgb="FF006100"/>
+      <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -999,7 +1000,7 @@
     <font>
       <b/>
       <sz val="11"/>
-      <color theme="1"/>
+      <color rgb="FF3F3F3F"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -1030,9 +1031,17 @@
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FF9C6500"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="15"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -1044,36 +1053,6 @@
     </font>
     <font>
       <b/>
-      <sz val="11"/>
-      <color rgb="FFFA7D00"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="13"/>
-      <color theme="3"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF3F3F3F"/>
-      <name val="Calibri"/>
-      <charset val="0"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <sz val="11"/>
       <color rgb="FFFA7D00"/>
       <name val="Calibri"/>
@@ -1097,9 +1076,30 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color rgb="FF9C6500"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <b/>
       <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
@@ -1169,7 +1169,49 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7"/>
+        <fgColor theme="9" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1181,7 +1223,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.799981688894314"/>
+        <fgColor theme="4" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1193,13 +1235,25 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
+        <fgColor theme="6" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1211,37 +1265,31 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.599993896298105"/>
+        <fgColor theme="6" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.799981688894314"/>
+        <fgColor theme="8" tint="0.599993896298105"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.599993896298105"/>
+        <fgColor theme="4"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.399975585192419"/>
+        <fgColor theme="5"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.599993896298105"/>
+        <fgColor theme="8" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1259,61 +1307,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFCC99"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="4"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF2F2F2"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.599993896298105"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="6" tint="0.399975585192419"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="9" tint="0.399975585192419"/>
+        <fgColor theme="5" tint="0.399975585192419"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1331,25 +1325,31 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9"/>
+        <fgColor rgb="FFC6EFCE"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="8"/>
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="4" tint="0.799981688894314"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFA5A5A5"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1392,52 +1392,17 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color rgb="FFB2B2B2"/>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
       </left>
-      <right style="thin">
-        <color rgb="FFB2B2B2"/>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
       </right>
-      <top style="thin">
-        <color rgb="FFB2B2B2"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FFB2B2B2"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color theme="4"/>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
       </top>
       <bottom style="double">
-        <color theme="4"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color theme="4" tint="0.499984740745262"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF7F7F7F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF7F7F7F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF7F7F7F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF7F7F7F"/>
+        <color rgb="FF3F3F3F"/>
       </bottom>
       <diagonal/>
     </border>
@@ -1460,23 +1425,58 @@
       <left/>
       <right/>
       <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB2B2B2"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB2B2B2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF7F7F7F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF7F7F7F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF7F7F7F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF7F7F7F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
       <bottom style="double">
         <color rgb="FFFF8001"/>
       </bottom>
       <diagonal/>
     </border>
     <border>
-      <left style="double">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="double">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="double">
-        <color rgb="FF3F3F3F"/>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4"/>
       </top>
       <bottom style="double">
-        <color rgb="FF3F3F3F"/>
+        <color theme="4"/>
       </bottom>
       <diagonal/>
     </border>
@@ -1486,10 +1486,10 @@
     <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="19" fillId="26" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="22" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1498,133 +1498,133 @@
     <xf numFmtId="41" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="12" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="43" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="20" borderId="7" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="4" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="6" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="15" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="15" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="14" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="40" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="29" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="29" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="40" borderId="10" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="39" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="18" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -2457,7 +2457,7 @@
       </c>
       <c r="D4" s="38">
         <f>COUNTIFS('Unit Plan'!R5:R48,"&gt;0",'Unit Plan'!S5:S48,"&lt;&gt;Yes")</f>
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="5" ht="24" customHeight="1" spans="1:4">
@@ -2482,7 +2482,7 @@
       </c>
       <c r="B6" s="38">
         <f>COUNTIF('Unit Plan'!Q5:Q48,"Completed")</f>
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C6" s="36" t="s">
         <v>9</v>
@@ -2505,7 +2505,7 @@
       </c>
       <c r="D7" s="38">
         <f>IFERROR(AVERAGE('Unit Plan'!P5:P48),"")</f>
-        <v>177.931034481073</v>
+        <v>171.99999999837</v>
       </c>
     </row>
     <row r="8" ht="24" customHeight="1" spans="1:4">
@@ -2514,7 +2514,7 @@
       </c>
       <c r="B8" s="38">
         <f>COUNTIFS('Unit Plan'!C5:C48,"Exercise",'Unit Plan'!O5:O48,"&lt;&gt;")</f>
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C8" s="36" t="s">
         <v>13</v>
@@ -2546,7 +2546,7 @@
       </c>
       <c r="B10" s="39">
         <f>IF(B5=0,"",B6/B5)</f>
-        <v>0.954545454545455</v>
+        <v>0.977272727272727</v>
       </c>
       <c r="C10" s="36" t="s">
         <v>17</v>
@@ -5416,18 +5416,22 @@
         <f t="shared" si="0"/>
         <v/>
       </c>
-      <c r="N47" s="24"/>
-      <c r="O47" s="24"/>
-      <c r="P47" s="8" t="str">
+      <c r="N47" s="24">
+        <v>46171</v>
+      </c>
+      <c r="O47" s="24">
+        <v>46171</v>
+      </c>
+      <c r="P47" s="8">
         <f t="shared" si="1"/>
-        <v/>
+        <v>0</v>
       </c>
       <c r="Q47" s="30" t="s">
-        <v>30</v>
-      </c>
-      <c r="R47" s="28" t="str">
+        <v>21</v>
+      </c>
+      <c r="R47" s="28">
         <f t="shared" si="2"/>
-        <v/>
+        <v>46173</v>
       </c>
       <c r="S47" s="27" t="s">
         <v>82</v>
@@ -5518,11 +5522,11 @@
     <dataValidation type="list" allowBlank="1" sqref="Q5:Q48">
       <formula1>Protocol!$J$1:$J$5</formula1>
     </dataValidation>
+    <dataValidation type="list" allowBlank="1" sqref="S5:S48">
+      <formula1>"Yes,No"</formula1>
+    </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="T5:T48">
       <formula1>Protocol!$K$1:$K$5</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="S5:S48">
-      <formula1>"Yes,No"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>